<commit_message>
BOQ: add notes column + cumulative qty. Quotes: add fixed category buttons (fans, water units, heating, etc)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -475,16 +475,16 @@
         <v>הזמנות רכש — עדכון אחרי הוצאה</v>
       </c>
       <c r="C4" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="D4" t="str">
-        <v>לאפשר עריכת הזמנת רכש אחרי שיצאה. שמירה בפרויקט + מודול חדש "תשלומים לספקים" עם סנכרון דו-כיווני</v>
+        <v>מודול "תשלומים לספקים" חדש בסיידבר. מציג כל הזמנות מכל הפרויקטים, עריכה inline, פילטור לפי פרויקט/סטטוס, סיכומים. עריכה מכל מקום מעדכנת את אותה רשומה.</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>נוסף דף SupplierPayments + קישור בניווט</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
add vehicles module with expenses and document uploads
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -397,14 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="70.83203125" customWidth="1"/>
     <col min="5" max="5" width="50.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="6" max="6" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
         <v>בוצע</v>
       </c>
       <c r="D4" t="str">
-        <v>מודול "תשלומים לספקים" חדש בסיידבר. מציג כל הזמנות מכל הפרויקטים, עריכה inline, פילטור לפי פרויקט/סטטוס, סיכומים. עריכה מכל מקום מעדכנת את אותה רשומה.</v>
+        <v>מודול "תשלומים לספקים" חדש בסיידבר. מציג כל הזמנות מכל הפרויקטים, עריכה inline, סנכרון דו-כיווני.</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -647,9 +647,69 @@
         <v>תלוי בחיבור וואטסאפ (סעיף 2)</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>הערות בכתב כמויות</v>
+      </c>
+      <c r="C13" t="str">
+        <v>בוצע</v>
+      </c>
+      <c r="D13" t="str">
+        <v>נוספה עמודת הערות בטבלת כתב הכמויות. ניתן לכתוב הערה לכל שורה.</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>כמות מצטברת בכתב כמויות</v>
+      </c>
+      <c r="C14" t="str">
+        <v>בוצע</v>
+      </c>
+      <c r="D14" t="str">
+        <v>נוספה עמודת כמות מצטברת ליד אחוז הביצוע — מציגה כמה יחידות בוצעו בפועל.</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>כפתורי קטגוריות בהצעת מחיר</v>
+      </c>
+      <c r="C15" t="str">
+        <v>בוצע</v>
+      </c>
+      <c r="D15" t="str">
+        <v>נוספו כפתורים קבועים מתחת לספקים: מפוחים, יחידות מים, מערכות הלחה, חימום תת רצפתי, תעלות פח, גרילים, עבודה, משאבות, צילרים, ויטאות, בקרה. כפתורים שאין להם מחירון מסומנים כ"ריק".</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v>גם אם אין עכשיו מחירים — הכפתורים מוכנים לכשיוזן מחירון</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
save purchase orders to Firestore - viewable and editable in project + supplier payments
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -495,16 +495,16 @@
         <v>מודול רכבים</v>
       </c>
       <c r="C5" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="D5" t="str">
-        <v>מודול חדש: רשימת רכבים, שיוך לעובד, תזכורות טסט/ביטוח/שמן, דיווח דלק, יומן נסיעות</v>
+        <v>מודול מלא: רשימת רכבים, שיוך עובד, תוקף טסט+ביטוח עם התראות, קילומטראז, הוצאות (דלק/טיפול/ביטוח/קנס), העלאת מסמכים (רישיון/ביטוח/טסט/ליסינג). כרטיסי סיכום + התראות אוטומטיות.</v>
       </c>
       <c r="E5" t="str">
         <v/>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>נוסף דף Vehicles + ניווט בסיידבר</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
fix CSV export: clean descriptions, add cumulative totals, fix clause numbers
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -397,14 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="70.83203125" customWidth="1"/>
-    <col min="5" max="5" width="50.83203125" customWidth="1"/>
-    <col min="6" max="6" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="80.83203125" customWidth="1"/>
+    <col min="5" max="5" width="55.83203125" customWidth="1"/>
+    <col min="6" max="6" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,19 +472,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>הזמנות רכש — עדכון אחרי הוצאה</v>
+        <v>הזמנות רכש — שמירה ועריכה</v>
       </c>
       <c r="C4" t="str">
         <v>בוצע</v>
       </c>
       <c r="D4" t="str">
-        <v>מודול "תשלומים לספקים" חדש בסיידבר. מציג כל הזמנות מכל הפרויקטים, עריכה inline, סנכרון דו-כיווני.</v>
+        <v>כל הזמנת רכש נשמרת ב-Firestore. מוצגת בפרויקט (טאב רכש → "הזמנות רכש שמורות") וגם במודול תשלומי ספקים (טאב "הזמנות רכש"). ניתנת לעריכה בשני המקומות — סנכרון דו-כיווני.</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
-        <v>נוסף דף SupplierPayments + קישור בניווט</v>
+        <v>תוקן באג שהזמנות לא הופיעו אחרי יצירה</v>
       </c>
     </row>
     <row r="5">
@@ -504,7 +504,7 @@
         <v/>
       </c>
       <c r="F5" t="str">
-        <v>נוסף דף Vehicles + ניווט בסיידבר</v>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -512,19 +512,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>שירות — התממשקות ל-FIXUS</v>
+        <v>שירות — טופס קריאת שירות + FIXUS</v>
       </c>
       <c r="C6" t="str">
-        <v>ממתין ללקוח</v>
+        <v>טרם בוצע</v>
       </c>
       <c r="D6" t="str">
-        <v>כרגע קריאות השירות ב-FIXUS (fixus.co.il). אפשרויות: API, ייבוא CSV, או בנייה מאפס</v>
+        <v>צריך: 1) טופס קריאת שירות פנימי במערכת. 2) לבדוק אם FIXUS (fixus.co.il) נותנים API להתממשקות — אם כן, נמשוך קריאות אוטומטית. אם לא — ייבוא CSV או בנייה מאפס.</v>
       </c>
       <c r="E6" t="str">
-        <v>לשאול את יניר: יש API ב-FIXUS? או שנבנה מודול שירות בתוך המערכת?</v>
+        <v>לשאול את יניר: יש API ב-FIXUS? האם יש להם תמיכה טכנית שאפשר לדבר איתה?</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>הלקוח ביקש גם טופס קריאת שירות עצמאי</v>
       </c>
     </row>
     <row r="7">
@@ -658,7 +658,7 @@
         <v>בוצע</v>
       </c>
       <c r="D13" t="str">
-        <v>נוספה עמודת הערות בטבלת כתב הכמויות. ניתן לכתוב הערה לכל שורה.</v>
+        <v>נוספה עמודת הערות בטבלת כתב הכמויות.</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -678,7 +678,7 @@
         <v>בוצע</v>
       </c>
       <c r="D14" t="str">
-        <v>נוספה עמודת כמות מצטברת ליד אחוז הביצוע — מציגה כמה יחידות בוצעו בפועל.</v>
+        <v>נוספה עמודת כמות מצטברת ליד אחוז הביצוע.</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -698,18 +698,58 @@
         <v>בוצע</v>
       </c>
       <c r="D15" t="str">
-        <v>נוספו כפתורים קבועים מתחת לספקים: מפוחים, יחידות מים, מערכות הלחה, חימום תת רצפתי, תעלות פח, גרילים, עבודה, משאבות, צילרים, ויטאות, בקרה. כפתורים שאין להם מחירון מסומנים כ"ריק".</v>
+        <v>מפוחים, יחידות מים, מערכות הלחה, חימום תת רצפתי, תעלות פח, גרילים, עבודה, משאבות, צילרים, ויטאות, בקרה.</v>
       </c>
       <c r="E15" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>גם אם אין עכשיו מחירים — הכפתורים מוכנים לכשיוזן מחירון</v>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>תהליך גבייה — עדכון זרימה</v>
+      </c>
+      <c r="C16" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="D16" t="str">
+        <v>תהליך חדש: חשבון מצטבר לאישור → עדכון כמויות מאושרות → הפקת חשבונית/חשבון עסקה → אם חשבון עסקה: ממתינים לאישור הנהלת הלקוח → אחרי אישור: הפקת חשבונית מס → אישור קבלת תשלום → אפשרות לפצל תשלום: קרן עכשיו + מע"מ בחודש עוקב.</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v>הלקוח הסביר: לפעמים מחלקים תשלום לקרן + מע"מ לחודש עוקב</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>באג ייצוא CSV כתב כמויות</v>
+      </c>
+      <c r="C17" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="D17" t="str">
+        <v>בעיות: 1) תיאורים ארוכים נשברים על מספר שורות — newlines לא מטופלים. 2) "טקסט ארוך:" ו"הערות:" מופיעים כפרפיקס מיותר. 3) גרשיים כפולים — מופיע 4 גרשיים במקום 2. 4) פסיקים בתוך תיאור (,,,,) לא escaped. 5) סדר פריטים הפוך — כותרות מופיעות אחרי הפריטים שלהן. 6) שורת "*** ב ***" באמצע בלי הקשר. 7) גרש מיותר בתחילת מספר סעיף.</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v>באג קריטי — האקסל לא שמיש</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CSV: limit description length, clean formatting, add BOQ redesign task
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
@@ -732,24 +732,44 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>באג ייצוא CSV כתב כמויות</v>
+        <v>שינוי לוגיקת כתב כמויות</v>
       </c>
       <c r="C17" t="str">
         <v>טרם בוצע</v>
       </c>
       <c r="D17" t="str">
+        <v>לבנות כמו דמו קונסטרקטור: טבלה אחת (לא טאבים), כל החשבונות בעמודות, מצטבר+יתרה+אחוז ביצוע. כפתור "הוסף חיוב" לכל שורה. סיכום מצטבר בתחתית עם קיזוזים ומע"מ.</v>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v>אושר ע"י טליה</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>באג ייצוא CSV כתב כמויות</v>
+      </c>
+      <c r="C18" t="str">
+        <v>תוקן חלקית</v>
+      </c>
+      <c r="D18" t="str">
         <v>בעיות: 1) תיאורים ארוכים נשברים על מספר שורות — newlines לא מטופלים. 2) "טקסט ארוך:" ו"הערות:" מופיעים כפרפיקס מיותר. 3) גרשיים כפולים — מופיע 4 גרשיים במקום 2. 4) פסיקים בתוך תיאור (,,,,) לא escaped. 5) סדר פריטים הפוך — כותרות מופיעות אחרי הפריטים שלהן. 6) שורת "*** ב ***" באמצע בלי הקשר. 7) גרש מיותר בתחילת מספר סעיף.</v>
       </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
         <v>באג קריטי — האקסל לא שמיש</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
collection flow: new statuses, payment split (principal/VAT), fix project name in follow-up tasks
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -715,16 +715,16 @@
         <v>תהליך גבייה — עדכון זרימה</v>
       </c>
       <c r="C16" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="D16" t="str">
-        <v>תהליך חדש: חשבון מצטבר לאישור → עדכון כמויות מאושרות → הפקת חשבונית/חשבון עסקה → אם חשבון עסקה: ממתינים לאישור הנהלת הלקוח → אחרי אישור: הפקת חשבונית מס → אישור קבלת תשלום → אפשרות לפצל תשלום: קרן עכשיו + מע"מ בחודש עוקב.</v>
+        <v>תוקן: 1) סטטוסים חדשים: ממתין לאישור הלקוח, חשבונית מס הופקה, שולם חלקי קרן. 2) תשלום חלקי: אפשרות לבחור קרן/מע"מ/חלקי — קרן מחשבת אוטומטית סכום ללא מע"מ ויוצרת משימת המשך על המע"מ לחודש עוקב. 3) שם פרויקט ולקוח נשמרים נכון במשימת המשך. 4) סרגל התקדמות בכתב כמויות עודכן ל-6 שלבים.</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>הלקוח הסביר: לפעמים מחלקים תשלום לקרן + מע"מ לחודש עוקב</v>
+        <v>באגים שתוקנו: שם לקוח חסר, invoice_number לא ברור, project_id לא מועבר</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
fix: dashboard purchase link, quote status, collection KPI clicks, vehicle edit form
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -397,14 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:H27"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="36.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="80.83203125" customWidth="1"/>
-    <col min="5" max="5" width="55.83203125" customWidth="1"/>
-    <col min="6" max="6" width="55.83203125" customWidth="1"/>
+    <col min="2" max="2" width="8.83203125" customWidth="1"/>
+    <col min="3" max="3" width="7.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="80.83203125" customWidth="1"/>
+    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+    <col min="8" max="8" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -412,18 +414,24 @@
         <v>#</v>
       </c>
       <c r="B1" t="str">
+        <v>מקור</v>
+      </c>
+      <c r="C1" t="str">
+        <v>תאריך</v>
+      </c>
+      <c r="D1" t="str">
         <v>נושא</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>סטטוס</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>פירוט</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>מה צריך מהלקוח</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>הערות</v>
       </c>
     </row>
@@ -432,19 +440,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C2" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D2" t="str">
         <v>יוזרים פשוטים</v>
       </c>
-      <c r="C2" t="str">
+      <c r="E2" t="str">
         <v>בוצע</v>
       </c>
-      <c r="D2" t="str">
-        <v>מערכת login עם שם + סיסמה בלבד, בלי אימייל. נשמר ב-Firestore.</v>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
       <c r="F2" t="str">
-        <v>yanir/yanir123, chaya/chaya123, dvora/dvora123, rivka/rivka123, shai/shai123, yehuda/yehuda123</v>
+        <v>מערכת login עם שם + סיסמה בלבד, בלי אימייל.</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>yanir/yanir123, shai/shai123, chaya/chaya123, dvora/dvora123, rivka/rivka123, yehuda/yehuda123. יניר ושי = admin, השאר = user. ההבדל: admin רואה הכל, user רואה רק מה ששויך אליו (כרגע אין הגבלה פעילה).</v>
       </c>
     </row>
     <row r="3">
@@ -452,19 +466,25 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>וואטסאפ — חיבור בוט</v>
+        <v>טליה</v>
       </c>
       <c r="C3" t="str">
-        <v>ממתין ללקוח</v>
+        <v>7.5</v>
       </c>
       <c r="D3" t="str">
-        <v>בוט וואטסאפ מוכן בקוד, חסרים פרטי חיבור</v>
+        <v>הזמנות רכש — שמירה ועריכה</v>
       </c>
       <c r="E3" t="str">
-        <v>יניר צריך להעביר: מספר טלפון עסקי + גישה ל-Meta Business Suite, או פשוט מספר טלפון וסורקים QR</v>
+        <v>בוצע</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>כל הזמנת רכש נשמרת. מוצגת בפרויקט + במודול תשלומי ספקים. סנכרון דו-כיווני.</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>תוקן באג שהזמנות לא הופיעו אחרי יצירה</v>
       </c>
     </row>
     <row r="4">
@@ -472,19 +492,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>הזמנות רכש — שמירה ועריכה</v>
+        <v>טליה</v>
       </c>
       <c r="C4" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D4" t="str">
+        <v>מודול רכבים</v>
+      </c>
+      <c r="E4" t="str">
         <v>בוצע</v>
       </c>
-      <c r="D4" t="str">
-        <v>כל הזמנת רכש נשמרת ב-Firestore. מוצגת בפרויקט (טאב רכש → "הזמנות רכש שמורות") וגם במודול תשלומי ספקים (טאב "הזמנות רכש"). ניתנת לעריכה בשני המקומות — סנכרון דו-כיווני.</v>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
       <c r="F4" t="str">
-        <v>תוקן באג שהזמנות לא הופיעו אחרי יצירה</v>
+        <v>רשימת רכבים, שיוך עובד, טסט+ביטוח+שמן, הוצאות, מסמכים.</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -492,18 +518,24 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>מודול רכבים</v>
+        <v>טליה</v>
       </c>
       <c r="C5" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D5" t="str">
+        <v>הערות + כמות מצטברת בכתב כמויות</v>
+      </c>
+      <c r="E5" t="str">
         <v>בוצע</v>
       </c>
-      <c r="D5" t="str">
-        <v>מודול מלא: רשימת רכבים, שיוך עובד, תוקף טסט+ביטוח עם התראות, קילומטראז, הוצאות (דלק/טיפול/ביטוח/קנס), העלאת מסמכים (רישיון/ביטוח/טסט/ליסינג). כרטיסי סיכום + התראות אוטומטיות.</v>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
       <c r="F5" t="str">
+        <v>נוספו עמודות הערות וכמות מצטברת בטבלת כתב הכמויות.</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
         <v/>
       </c>
     </row>
@@ -512,19 +544,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>שירות — טופס קריאת שירות + FIXUS</v>
+        <v>טליה</v>
       </c>
       <c r="C6" t="str">
-        <v>טרם בוצע</v>
+        <v>7.5</v>
       </c>
       <c r="D6" t="str">
-        <v>צריך: 1) טופס קריאת שירות פנימי במערכת. 2) לבדוק אם FIXUS (fixus.co.il) נותנים API להתממשקות — אם כן, נמשוך קריאות אוטומטית. אם לא — ייבוא CSV או בנייה מאפס.</v>
+        <v>כפתורי קטגוריות בהצעת מחיר</v>
       </c>
       <c r="E6" t="str">
-        <v>לשאול את יניר: יש API ב-FIXUS? האם יש להם תמיכה טכנית שאפשר לדבר איתה?</v>
+        <v>בוצע</v>
       </c>
       <c r="F6" t="str">
-        <v>הלקוח ביקש גם טופס קריאת שירות עצמאי</v>
+        <v>מפוחים, יחידות מים, מערכות הלחה, חימום תת רצפתי, תעלות פח, גרילים, עבודה, משאבות, צילרים, ויטאות, בקרה.</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -532,19 +570,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>אקסלים של רבקה</v>
+        <v>טליה</v>
       </c>
       <c r="C7" t="str">
-        <v>ממתין ללקוח</v>
+        <v>8.5</v>
       </c>
       <c r="D7" t="str">
-        <v>לבנות ממשק מסודר במערכת במקום האקסלים</v>
+        <v>תהליך גבייה — עדכון זרימה</v>
       </c>
       <c r="E7" t="str">
-        <v>לבקש מרבקה את כל האקסלים שהיא עובדת איתם</v>
+        <v>בוצע</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>סטטוסים חדשים: ממתין לאישור הלקוח, חשבונית מס הופקה, שולם חלקי קרן. תשלום חלקי: קרן/מע"מ/חלקי. סרגל 6 שלבים.</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>תוקן: שם לקוח חסר במשימת המשך, project_id לא מועבר</v>
       </c>
     </row>
     <row r="8">
@@ -552,19 +596,25 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>בקשות תשלום</v>
+        <v>טליה</v>
       </c>
       <c r="C8" t="str">
-        <v>טרם בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D8" t="str">
-        <v>שליחת בקשת תשלום ממותגת עם לוגו + אפשרות צירוף קובץ. שליחה במייל/וואטסאפ. מעקב סטטוס</v>
+        <v>ייצוא אקסל XLSX (לא CSV)</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>בוצע</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>ייצוא כתב כמויות כ-XLSX מעוצב: RTL, כותרת כחולה, רוחב עמודות, סיכום מצטבר, גרסה עם/בלי מחירים.</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>בלי מחירים = אחוזי ביצוע + כמות שבוצעה + כמות שנותרה</v>
       </c>
     </row>
     <row r="9">
@@ -572,18 +622,24 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>חשבונות חלקיים</v>
+        <v>יניר</v>
       </c>
       <c r="C9" t="str">
-        <v>טרם בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D9" t="str">
-        <v>בתוך פרויקט — כפתור "חשבון חלקי", בחירת אחוז/סכום, PDF ממותג, מעקב כמה חויב וכמה נשאר</v>
+        <v>משימות — סינון לפי פרויקט</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F9" t="str">
+        <v>במרכז המשימות להוסיף אפשרות סינון לפי פרויקט.</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
         <v/>
       </c>
     </row>
@@ -592,18 +648,24 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>קבלני משנה</v>
+        <v>יניר</v>
       </c>
       <c r="C10" t="str">
-        <v>טרם בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D10" t="str">
-        <v>מודול ניהול מרכזי: רשימה, שיוך לפרויקט, מעקב תשלומים, הזמנת עבודה PDF</v>
+        <v>דשבורד — כפתור רכש מוביל למקום לא נכון</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F10" t="str">
+        <v>כפתור רכש בלוח בקרה לוקח לרשימת פרויקטים במקום להזמנות רכש. צריך לקשר למודול תשלומי ספקים.</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
         <v/>
       </c>
     </row>
@@ -612,19 +674,25 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>התראות עיקבון לגבייה</v>
+        <v>יניר</v>
       </c>
       <c r="C11" t="str">
-        <v>טרם בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D11" t="str">
-        <v>כשפרויקט מסתיים ויש עיקבון — התראה עתידית (גם שנה-שנתיים). שליחה בוואטסאפ + במערכת</v>
+        <v>הצעת מחיר — סוג מסחרי/פרטי</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>לבחור אם הצעה מסחרית או פרטית. בפרטי — ה-PDF יצא עם מסמכים נוספים: אודות החברה + הסבר על המערכת.</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>שאלה: האם יש PDF מוכן של אודות החברה? או שצריך לבנות?</v>
       </c>
     </row>
     <row r="12">
@@ -632,19 +700,25 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>משימות קבועות בוואטסאפ</v>
+        <v>יניר</v>
       </c>
       <c r="C12" t="str">
-        <v>טרם בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D12" t="str">
-        <v>הגדרת משימות חוזרות (חודשי) לאנשים ספציפיים. דוגמה: לעבור על פרויקטים ישנים, לסגור הצעות מחיר</v>
+        <v>הצעת מחיר — שינוי סטטוס לא עובד</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F12" t="str">
-        <v>תלוי בחיבור וואטסאפ (סעיף 2)</v>
+        <v>ברשימת הצעות המחיר לא ניתן לשנות סטטוס הצעה.</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -652,18 +726,24 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>הערות בכתב כמויות</v>
+        <v>יניר</v>
       </c>
       <c r="C13" t="str">
-        <v>בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D13" t="str">
-        <v>נוספה עמודת הערות בטבלת כתב הכמויות.</v>
+        <v>דשבורד גבייה — כפתורי KPI לא לוחצים</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F13" t="str">
+        <v>כפתורים בדשבורד גבייה הם רק תצוגה. צריך: לחיצה על "כספים באיחור" → רשימת המאחרים. "שולם השבוע" → מי שילם ומתי.</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
         <v/>
       </c>
     </row>
@@ -672,18 +752,24 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>כמות מצטברת בכתב כמויות</v>
+        <v>יניר</v>
       </c>
       <c r="C14" t="str">
-        <v>בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D14" t="str">
-        <v>נוספה עמודת כמות מצטברת ליד אחוז הביצוע.</v>
+        <v>תשלומי ספקים — חסר תיאור פריט + סכום כולל</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F14" t="str">
+        <v>במודול תשלומי ספקים: 1) חסר חישוב סכום כולל. 2) חסר תיאור פריט — רואים סכום בלי לדעת מה זה. 3) לחיצה מעבירה לפרויקט ולא לפריט בכתב כמויות.</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
         <v/>
       </c>
     </row>
@@ -692,18 +778,24 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>כפתורי קטגוריות בהצעת מחיר</v>
+        <v>יניר</v>
       </c>
       <c r="C15" t="str">
-        <v>בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D15" t="str">
-        <v>מפוחים, יחידות מים, מערכות הלחה, חימום תת רצפתי, תעלות פח, גרילים, עבודה, משאבות, צילרים, ויטאות, בקרה.</v>
+        <v>רכבים — התראות בדשבורד הראשי</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F15" t="str">
+        <v>התראות רכבים (טסט/ביטוח) שיופיעו גם בדשבורד הראשי ולא רק במודול רכבים.</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
         <v/>
       </c>
     </row>
@@ -712,19 +804,25 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>תהליך גבייה — עדכון זרימה</v>
+        <v>יניר</v>
       </c>
       <c r="C16" t="str">
-        <v>בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D16" t="str">
-        <v>תוקן: 1) סטטוסים חדשים: ממתין לאישור הלקוח, חשבונית מס הופקה, שולם חלקי קרן. 2) תשלום חלקי: אפשרות לבחור קרן/מע"מ/חלקי — קרן מחשבת אוטומטית סכום ללא מע"מ ויוצרת משימת המשך על המע"מ לחודש עוקב. 3) שם פרויקט ולקוח נשמרים נכון במשימת המשך. 4) סרגל התקדמות בכתב כמויות עודכן ל-6 שלבים.</v>
+        <v>רכבים — עריכה לא מציגה פרטים</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>טרם בוצע</v>
       </c>
       <c r="F16" t="str">
-        <v>באגים שתוקנו: שם לקוח חסר, invoice_number לא ברור, project_id לא מועבר</v>
+        <v>כשפותחים עריכה של רכב קיים, הפרטים הקיימים לא מופיעים בטופס.</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -732,19 +830,25 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>שינוי לוגיקת כתב כמויות</v>
+        <v>יניר</v>
       </c>
       <c r="C17" t="str">
-        <v>טרם בוצע</v>
+        <v>8.5</v>
       </c>
       <c r="D17" t="str">
-        <v>לבנות כמו דמו קונסטרקטור: טבלה אחת (לא טאבים), כל החשבונות בעמודות, מצטבר+יתרה+אחוז ביצוע. כפתור "הוסף חיוב" לכל שורה. סיכום מצטבר בתחתית עם קיזוזים ומע"מ.</v>
+        <v>רכבים — דיווח ק"מ שבועי</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>שאלה</v>
       </c>
       <c r="F17" t="str">
-        <v>אושר ע"י טליה</v>
+        <v>האם דיווח קילומטראז שבועי ידני (חיה מזינה) או אוטומטי (העובד מדווח)?</v>
+      </c>
+      <c r="G17" t="str">
+        <v>יניר — לענות</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -752,24 +856,264 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>באג ייצוא CSV כתב כמויות</v>
+        <v>יניר</v>
       </c>
       <c r="C18" t="str">
-        <v>תוקן חלקית</v>
+        <v>8.5</v>
       </c>
       <c r="D18" t="str">
-        <v>בעיות: 1) תיאורים ארוכים נשברים על מספר שורות — newlines לא מטופלים. 2) "טקסט ארוך:" ו"הערות:" מופיעים כפרפיקס מיותר. 3) גרשיים כפולים — מופיע 4 גרשיים במקום 2. 4) פסיקים בתוך תיאור (,,,,) לא escaped. 5) סדר פריטים הפוך — כותרות מופיעות אחרי הפריטים שלהן. 6) שורת "*** ב ***" באמצע בלי הקשר. 7) גרש מיותר בתחילת מספר סעיף.</v>
+        <v>דוחות כספיים</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>ממתין ללקוח</v>
       </c>
       <c r="F18" t="str">
-        <v>באג קריטי — האקסל לא שמיש</v>
+        <v>יניר ישלח קבצים. לבנות דוחות כספיים במערכת.</v>
+      </c>
+      <c r="G18" t="str">
+        <v>יניר — לשלוח קבצים</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>יניר</v>
+      </c>
+      <c r="C19" t="str">
+        <v>8.5</v>
+      </c>
+      <c r="D19" t="str">
+        <v>הבדל admin/user + טבלת יוזרים</v>
+      </c>
+      <c r="E19" t="str">
+        <v>שאלה</v>
+      </c>
+      <c r="F19" t="str">
+        <v>יניר שאל מה ההבדל. כרגע: admin = יניר+שי, user = חיה+דבורה+רבקה+יהודה. אין הגבלות פעילות — כולם רואים הכל.</v>
+      </c>
+      <c r="G19" t="str">
+        <v>יניר — האם רוצה הגבלות? מה user לא אמור לראות?</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C20" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D20" t="str">
+        <v>וואטסאפ — חיבור בוט</v>
+      </c>
+      <c r="E20" t="str">
+        <v>ממתין ללקוח</v>
+      </c>
+      <c r="F20" t="str">
+        <v>בוט מוכן, חסרים פרטי חיבור.</v>
+      </c>
+      <c r="G20" t="str">
+        <v>יניר — מספר טלפון עסקי + גישה ל-Meta Business Suite</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C21" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D21" t="str">
+        <v>שירות — טופס + FIXUS</v>
+      </c>
+      <c r="E21" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F21" t="str">
+        <v>טופס קריאת שירות + בדיקת התממשקות FIXUS.</v>
+      </c>
+      <c r="G21" t="str">
+        <v>יניר — יש API ב-FIXUS?</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C22" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D22" t="str">
+        <v>אקסלים של רבקה</v>
+      </c>
+      <c r="E22" t="str">
+        <v>ממתין ללקוח</v>
+      </c>
+      <c r="F22" t="str">
+        <v>לבנות ממשק במערכת במקום אקסלים.</v>
+      </c>
+      <c r="G22" t="str">
+        <v>רבקה — לשלוח את האקסלים</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C23" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D23" t="str">
+        <v>בקשות תשלום ממותגות</v>
+      </c>
+      <c r="E23" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F23" t="str">
+        <v>שליחת בקשת תשלום עם לוגו + צירוף קובץ.</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C24" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D24" t="str">
+        <v>קבלני משנה — מודול</v>
+      </c>
+      <c r="E24" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F24" t="str">
+        <v>מודול ניהול מרכזי: רשימה, שיוך לפרויקט, מעקב תשלומים.</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C25" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D25" t="str">
+        <v>התראות עיקבון לגבייה</v>
+      </c>
+      <c r="E25" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F25" t="str">
+        <v>התראה כשפרויקט מסתיים ויש עיקבון (גם שנה-שנתיים).</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C26" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D26" t="str">
+        <v>משימות קבועות בוואטסאפ</v>
+      </c>
+      <c r="E26" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F26" t="str">
+        <v>משימות חוזרות חודשיות לאנשים ספציפיים.</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v>תלוי בחיבור וואטסאפ</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C27" t="str">
+        <v>8.5</v>
+      </c>
+      <c r="D27" t="str">
+        <v>שינוי לוגיקת כתב כמויות</v>
+      </c>
+      <c r="E27" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F27" t="str">
+        <v>טבלה אחת (לא טאבים), כל החשבונות בעמודות. אושר ע"י טליה.</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
tasks: project filter, supplier payments: item desc + totals, dashboard: vehicle alerts
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -657,10 +657,10 @@
         <v>דשבורד — כפתור רכש מוביל למקום לא נכון</v>
       </c>
       <c r="E10" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F10" t="str">
-        <v>כפתור רכש בלוח בקרה לוקח לרשימת פרויקטים במקום להזמנות רכש. צריך לקשר למודול תשלומי ספקים.</v>
+        <v>תוקן: כפתור רכש בדשבורד מוביל עכשיו למודול תשלומי ספקים.</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -709,16 +709,16 @@
         <v>הצעת מחיר — שינוי סטטוס לא עובד</v>
       </c>
       <c r="E12" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F12" t="str">
-        <v>ברשימת הצעות המחיר לא ניתן לשנות סטטוס הצעה.</v>
+        <v>תוקן: נוסף dropdown לשינוי סטטוס בדף הצעות המחיר. שינוי ל"אושרה" מפעיל את אותה זרימה כמו אישור ליד — מעדכן את הליד ל"אושר" ויוצר פרויקט חדש אוטומטית. אפשר לאשר גם מהליד וגם מההצעה — התוצאה זהה.</v>
       </c>
       <c r="G12" t="str">
         <v/>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>ליניר: אפשר לאשר הצעה מ-2 מקומות: 1) מדף הלידים → שינוי סטטוס ל"אושר" 2) מדף הצעות המחיר → שינוי סטטוס ל"אושרה". בשני המקרים נפתח פרויקט אוטומטית.</v>
       </c>
     </row>
     <row r="13">
@@ -735,10 +735,10 @@
         <v>דשבורד גבייה — כפתורי KPI לא לוחצים</v>
       </c>
       <c r="E13" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F13" t="str">
-        <v>כפתורים בדשבורד גבייה הם רק תצוגה. צריך: לחיצה על "כספים באיחור" → רשימת המאחרים. "שולם השבוע" → מי שילם ומתי.</v>
+        <v>תוקן: לחיצה על "כספים באיחור" / "שולם השבוע" / "שולם החודש" פותחת דיאלוג עם טבלה מפורטת — פרויקט, סכום, ימי איחור/תאריך, סטטוס.</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -813,10 +813,10 @@
         <v>רכבים — עריכה לא מציגה פרטים</v>
       </c>
       <c r="E16" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F16" t="str">
-        <v>כשפותחים עריכה של רכב קיים, הפרטים הקיימים לא מופיעים בטופס.</v>
+        <v>תוקן: פרטי הרכב הקיים מופיעים עכשיו בטופס העריכה.</v>
       </c>
       <c r="G16" t="str">
         <v/>

</xml_diff>

<commit_message>
update tracker: items 8,13,14 done
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -631,10 +631,10 @@
         <v>משימות — סינון לפי פרויקט</v>
       </c>
       <c r="E9" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F9" t="str">
-        <v>במרכז המשימות להוסיף אפשרות סינון לפי פרויקט.</v>
+        <v>נוסף dropdown סינון לפי פרויקט בדף המשימות.</v>
       </c>
       <c r="G9" t="str">
         <v/>
@@ -761,10 +761,10 @@
         <v>תשלומי ספקים — חסר תיאור פריט + סכום כולל</v>
       </c>
       <c r="E14" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F14" t="str">
-        <v>במודול תשלומי ספקים: 1) חסר חישוב סכום כולל. 2) חסר תיאור פריט — רואים סכום בלי לדעת מה זה. 3) לחיצה מעבירה לפרויקט ולא לפריט בכתב כמויות.</v>
+        <v>תוקן: 1) תיאור פריט מוצג מתחת לשם. 2) סכום כולל בתחתית הטבלה. 3) לחיצה על פרויקט מנווטת לטאב רכש.</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -787,10 +787,10 @@
         <v>רכבים — התראות בדשבורד הראשי</v>
       </c>
       <c r="E15" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F15" t="str">
-        <v>התראות רכבים (טסט/ביטוח) שיופיעו גם בדשבורד הראשי ולא רק במודול רכבים.</v>
+        <v>תוקן: התראות רכבים (טסט/ביטוח שפג או עומד לפוג ב-30 יום) מופיעות עכשיו בדשבורד הראשי.</v>
       </c>
       <c r="G15" t="str">
         <v/>

</xml_diff>

<commit_message>
add subcontractors central module with filters, edit, totals
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -1021,10 +1021,10 @@
         <v>קבלני משנה — מודול</v>
       </c>
       <c r="E24" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F24" t="str">
-        <v>מודול ניהול מרכזי: רשימה, שיוך לפרויקט, מעקב תשלומים.</v>
+        <v>מודול מרכזי בסיידבר: כל קבלני המשנה מכל הפרויקטים, פילטור לפי פרויקט/תחום/סטטוס, עריכה inline, סיכומים (סה"כ/שולם/ממתין), לינק לפרויקט.</v>
       </c>
       <c r="G24" t="str">
         <v/>

</xml_diff>

<commit_message>
retention alerts: auto-create task when project completed with retention period, subcontractors module
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -1047,10 +1047,10 @@
         <v>התראות עיקבון לגבייה</v>
       </c>
       <c r="E25" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F25" t="str">
-        <v>התראה כשפרויקט מסתיים ויש עיקבון (גם שנה-שנתיים).</v>
+        <v>בכל פרויקט יש שדה "עיקבון (חודשים)" בכותרת. כשהפרויקט עובר ל"הושלם" — נוצרת משימה אוטומטית לרבקה עם תאריך יעד לפי תקופת העיקבון. גם 12 חודשים, גם 24 — הכל עובד.</v>
       </c>
       <c r="G25" t="str">
         <v/>

</xml_diff>

<commit_message>
update tracker with all completed items through 12.5
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/argaman-requests.xlsx
+++ b/argaman-requests.xlsx
@@ -397,15 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H29"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
     <col min="3" max="3" width="7.83203125" customWidth="1"/>
-    <col min="4" max="4" width="38.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
     <col min="6" max="6" width="80.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
     <col min="8" max="8" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -458,7 +458,7 @@
         <v/>
       </c>
       <c r="H2" t="str">
-        <v>yanir/yanir123, shai/shai123, chaya/chaya123, dvora/dvora123, rivka/rivka123, yehuda/yehuda123. יניר ושי = admin, השאר = user. ההבדל: admin רואה הכל, user רואה רק מה ששויך אליו (כרגע אין הגבלה פעילה).</v>
+        <v>yanir/yanir123, shai/shai123, chaya/chaya123, dvora/dvora123, rivka/rivka123, yehuda/yehuda123. יניר ושי = admin, השאר = user.</v>
       </c>
     </row>
     <row r="3">
@@ -582,7 +582,7 @@
         <v>בוצע</v>
       </c>
       <c r="F7" t="str">
-        <v>סטטוסים חדשים: ממתין לאישור הלקוח, חשבונית מס הופקה, שולם חלקי קרן. תשלום חלקי: קרן/מע"מ/חלקי. סרגל 6 שלבים.</v>
+        <v>סטטוסים חדשים: ממתין לאישור הלקוח, חשבונית מס הופקה, שולם חלקי קרן. תשלום חלקי: קרן/מע"מ/חלקי עם חישוב אוטומטי. סרגל 6 שלבים.</v>
       </c>
       <c r="G7" t="str">
         <v/>
@@ -602,19 +602,19 @@
         <v>8.5</v>
       </c>
       <c r="D8" t="str">
-        <v>ייצוא אקסל XLSX (לא CSV)</v>
+        <v>ייצוא אקסל XLSX</v>
       </c>
       <c r="E8" t="str">
         <v>בוצע</v>
       </c>
       <c r="F8" t="str">
-        <v>ייצוא כתב כמויות כ-XLSX מעוצב: RTL, כותרת כחולה, רוחב עמודות, סיכום מצטבר, גרסה עם/בלי מחירים.</v>
+        <v>ייצוא כתב כמויות כ-XLSX מעוצב: RTL, כותרת כחולה, רוחב עמודות, סיכום מצטבר. בלי מחירים = אחוזי ביצוע + כמות שבוצעה + כמות שנותרה.</v>
       </c>
       <c r="G8" t="str">
         <v/>
       </c>
       <c r="H8" t="str">
-        <v>בלי מחירים = אחוזי ביצוע + כמות שבוצעה + כמות שנותרה</v>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -654,13 +654,13 @@
         <v>8.5</v>
       </c>
       <c r="D10" t="str">
-        <v>דשבורד — כפתור רכש מוביל למקום לא נכון</v>
+        <v>דשבורד — כפתור רכש</v>
       </c>
       <c r="E10" t="str">
         <v>בוצע</v>
       </c>
       <c r="F10" t="str">
-        <v>תוקן: כפתור רכש בדשבורד מוביל עכשיו למודול תשלומי ספקים.</v>
+        <v>תוקן: כפתור רכש בדשבורד מוביל למודול תשלומי ספקים.</v>
       </c>
       <c r="G10" t="str">
         <v/>
@@ -683,16 +683,16 @@
         <v>הצעת מחיר — סוג מסחרי/פרטי</v>
       </c>
       <c r="E11" t="str">
-        <v>טרם בוצע</v>
+        <v>בוצע</v>
       </c>
       <c r="F11" t="str">
-        <v>לבחור אם הצעה מסחרית או פרטית. בפרטי — ה-PDF יצא עם מסמכים נוספים: אודות החברה + הסבר על המערכת.</v>
+        <v>נוסף בורר מסחרי/פרטי בדף הצעת המחיר. בפרטי — יורד גם PDF אודות החברה יחד עם ההצעה.</v>
       </c>
       <c r="G11" t="str">
         <v/>
       </c>
       <c r="H11" t="str">
-        <v>שאלה: האם יש PDF מוכן של אודות החברה? או שצריך לבנות?</v>
+        <v>PDF אודות חברה התקבל מיניר והועלה למערכת</v>
       </c>
     </row>
     <row r="12">
@@ -706,19 +706,19 @@
         <v>8.5</v>
       </c>
       <c r="D12" t="str">
-        <v>הצעת מחיר — שינוי סטטוס לא עובד</v>
+        <v>הצעת מחיר — שינוי סטטוס + זרימה</v>
       </c>
       <c r="E12" t="str">
         <v>בוצע</v>
       </c>
       <c r="F12" t="str">
-        <v>תוקן: נוסף dropdown לשינוי סטטוס בדף הצעות המחיר. שינוי ל"אושרה" מפעיל את אותה זרימה כמו אישור ליד — מעדכן את הליד ל"אושר" ויוצר פרויקט חדש אוטומטית. אפשר לאשר גם מהליד וגם מההצעה — התוצאה זהה.</v>
+        <v>נוסף dropdown סטטוס. שינוי ל"אושרה" מפעיל אותה זרימה כמו אישור ליד — מעדכן ליד + יוצר פרויקט. אפשר לאשר מ-2 מקומות: מהליד או מההצעה.</v>
       </c>
       <c r="G12" t="str">
         <v/>
       </c>
       <c r="H12" t="str">
-        <v>ליניר: אפשר לאשר הצעה מ-2 מקומות: 1) מדף הלידים → שינוי סטטוס ל"אושר" 2) מדף הצעות המחיר → שינוי סטטוס ל"אושרה". בשני המקרים נפתח פרויקט אוטומטית.</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -732,13 +732,13 @@
         <v>8.5</v>
       </c>
       <c r="D13" t="str">
-        <v>דשבורד גבייה — כפתורי KPI לא לוחצים</v>
+        <v>דשבורד גבייה — כפתורי KPI</v>
       </c>
       <c r="E13" t="str">
         <v>בוצע</v>
       </c>
       <c r="F13" t="str">
-        <v>תוקן: לחיצה על "כספים באיחור" / "שולם השבוע" / "שולם החודש" פותחת דיאלוג עם טבלה מפורטת — פרויקט, סכום, ימי איחור/תאריך, סטטוס.</v>
+        <v>לחיצה על כספים באיחור/שולם השבוע/שולם החודש פותחת דיאלוג עם רשימה מפורטת.</v>
       </c>
       <c r="G13" t="str">
         <v/>
@@ -758,13 +758,13 @@
         <v>8.5</v>
       </c>
       <c r="D14" t="str">
-        <v>תשלומי ספקים — חסר תיאור פריט + סכום כולל</v>
+        <v>תשלומי ספקים — תיאור + סכום</v>
       </c>
       <c r="E14" t="str">
         <v>בוצע</v>
       </c>
       <c r="F14" t="str">
-        <v>תוקן: 1) תיאור פריט מוצג מתחת לשם. 2) סכום כולל בתחתית הטבלה. 3) לחיצה על פרויקט מנווטת לטאב רכש.</v>
+        <v>תיאור פריט מוצג מתחת לשם. סכום כולל בתחתית. לחיצה מנווטת לטאב רכש בפרויקט.</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -784,13 +784,13 @@
         <v>8.5</v>
       </c>
       <c r="D15" t="str">
-        <v>רכבים — התראות בדשבורד הראשי</v>
+        <v>רכבים — התראות בדשבורד</v>
       </c>
       <c r="E15" t="str">
         <v>בוצע</v>
       </c>
       <c r="F15" t="str">
-        <v>תוקן: התראות רכבים (טסט/ביטוח שפג או עומד לפוג ב-30 יום) מופיעות עכשיו בדשבורד הראשי.</v>
+        <v>התראות טסט/ביטוח מופיעות בדשבורד הראשי.</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -816,7 +816,7 @@
         <v>בוצע</v>
       </c>
       <c r="F16" t="str">
-        <v>תוקן: פרטי הרכב הקיים מופיעים עכשיו בטופס העריכה.</v>
+        <v>תוקן: פרטי הרכב מופיעים בטופס העריכה.</v>
       </c>
       <c r="G16" t="str">
         <v/>
@@ -830,22 +830,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>יניר</v>
+        <v>טליה</v>
       </c>
       <c r="C17" t="str">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="D17" t="str">
-        <v>רכבים — דיווח ק"מ שבועי</v>
+        <v>קבלני משנה — מודול מרכזי</v>
       </c>
       <c r="E17" t="str">
-        <v>שאלה</v>
+        <v>בוצע</v>
       </c>
       <c r="F17" t="str">
-        <v>האם דיווח קילומטראז שבועי ידני (חיה מזינה) או אוטומטי (העובד מדווח)?</v>
+        <v>מודול בסיידבר: כל קבלני המשנה מכל הפרויקטים, פילטור לפי פרויקט/תחום/סטטוס, עריכה inline, סיכומים.</v>
       </c>
       <c r="G17" t="str">
-        <v>יניר — לענות</v>
+        <v/>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -856,22 +856,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>יניר</v>
+        <v>טליה</v>
       </c>
       <c r="C18" t="str">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="D18" t="str">
-        <v>דוחות כספיים</v>
+        <v>התראות עיקבון לגבייה</v>
       </c>
       <c r="E18" t="str">
-        <v>ממתין ללקוח</v>
+        <v>בוצע</v>
       </c>
       <c r="F18" t="str">
-        <v>יניר ישלח קבצים. לבנות דוחות כספיים במערכת.</v>
+        <v>שדה "עיקבון (חודשים)" בכל פרויקט. כשפרויקט הושלם — משימה אוטומטית לרבקה עם תאריך יעד.</v>
       </c>
       <c r="G18" t="str">
-        <v>יניר — לשלוח קבצים</v>
+        <v/>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -885,22 +885,22 @@
         <v>יניר</v>
       </c>
       <c r="C19" t="str">
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="D19" t="str">
-        <v>הבדל admin/user + טבלת יוזרים</v>
+        <v>דיווח ק"מ חודשי</v>
       </c>
       <c r="E19" t="str">
-        <v>שאלה</v>
+        <v>בוצע</v>
       </c>
       <c r="F19" t="str">
-        <v>יניר שאל מה ההבדל. כרגע: admin = יניר+שי, user = חיה+דבורה+רבקה+יהודה. אין הגבלות פעילות — כולם רואים הכל.</v>
+        <v>דף ציבורי בלי login: argaman-new.vercel.app/KmReport — מציג כל הרכבים, מזינים ק"מ ושולחים. לינק נשלח פעם בחודש.</v>
       </c>
       <c r="G19" t="str">
-        <v>יניר — האם רוצה הגבלות? מה user לא אמור לראות?</v>
+        <v/>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>יניר אמר: דיווח דרך יומן עבודה, פעם בחודש. בנינו דף ציבורי שנשלח כלינק</v>
       </c>
     </row>
     <row r="20">
@@ -908,22 +908,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>טליה</v>
+        <v>יניר</v>
       </c>
       <c r="C20" t="str">
-        <v>7.5</v>
+        <v>12.5</v>
       </c>
       <c r="D20" t="str">
-        <v>וואטסאפ — חיבור בוט</v>
+        <v>הצעת מחיר — PDF אודות חברה</v>
       </c>
       <c r="E20" t="str">
-        <v>ממתין ללקוח</v>
+        <v>בוצע</v>
       </c>
       <c r="F20" t="str">
-        <v>בוט מוכן, חסרים פרטי חיבור.</v>
+        <v>יניר שלח PDF אודות. הועלה למערכת. בהצעה פרטית יורד אוטומטית יחד עם ההצעה.</v>
       </c>
       <c r="G20" t="str">
-        <v>יניר — מספר טלפון עסקי + גישה ל-Meta Business Suite</v>
+        <v/>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -934,22 +934,22 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>טליה</v>
+        <v>יניר</v>
       </c>
       <c r="C21" t="str">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="D21" t="str">
-        <v>שירות — טופס + FIXUS</v>
+        <v>דוחות כספיים</v>
       </c>
       <c r="E21" t="str">
-        <v>טרם בוצע</v>
+        <v>ממתין ללקוח</v>
       </c>
       <c r="F21" t="str">
-        <v>טופס קריאת שירות + בדיקת התממשקות FIXUS.</v>
+        <v>יניר אמר שישלח קבצים.</v>
       </c>
       <c r="G21" t="str">
-        <v>יניר — יש API ב-FIXUS?</v>
+        <v>יניר — לשלוח קבצים</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -960,22 +960,22 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>טליה</v>
+        <v>יניר</v>
       </c>
       <c r="C22" t="str">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="D22" t="str">
-        <v>אקסלים של רבקה</v>
+        <v>הרשאות admin/user</v>
       </c>
       <c r="E22" t="str">
         <v>ממתין ללקוח</v>
       </c>
       <c r="F22" t="str">
-        <v>לבנות ממשק במערכת במקום אקסלים.</v>
+        <v>כרגע כולם רואים הכל. שאלנו מה user לא אמור לראות.</v>
       </c>
       <c r="G22" t="str">
-        <v>רבקה — לשלוח את האקסלים</v>
+        <v>יניר — לענות</v>
       </c>
       <c r="H22" t="str">
         <v/>
@@ -986,25 +986,25 @@
         <v>22</v>
       </c>
       <c r="B23" t="str">
-        <v>טליה</v>
+        <v>יניר</v>
       </c>
       <c r="C23" t="str">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
       <c r="D23" t="str">
-        <v>בקשות תשלום ממותגות</v>
+        <v>משימות אוטומטיות — אישור רלוונטיות</v>
       </c>
       <c r="E23" t="str">
-        <v>טרם בוצע</v>
+        <v>ממתין ללקוח</v>
       </c>
       <c r="F23" t="str">
-        <v>שליחת בקשת תשלום עם לוגו + צירוף קובץ.</v>
+        <v>שלחנו ליניר רשימה של כל המשימות האוטומטיות לאישור.</v>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>יניר — לאשר</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>נשלח במסמך שאלות-ליניר</v>
       </c>
     </row>
     <row r="24">
@@ -1018,19 +1018,19 @@
         <v>7.5</v>
       </c>
       <c r="D24" t="str">
-        <v>קבלני משנה — מודול</v>
+        <v>וואטסאפ — חיבור בוט</v>
       </c>
       <c r="E24" t="str">
-        <v>בוצע</v>
+        <v>ממתין ללקוח</v>
       </c>
       <c r="F24" t="str">
-        <v>מודול מרכזי בסיידבר: כל קבלני המשנה מכל הפרויקטים, פילטור לפי פרויקט/תחום/סטטוס, עריכה inline, סיכומים (סה"כ/שולם/ממתין), לינק לפרויקט.</v>
+        <v>בוט מוכן. יניר אמר שקונים סים חדש.</v>
       </c>
       <c r="G24" t="str">
-        <v/>
+        <v>יניר — לקנות סים חדש, להתקין וואטסאפ, לשלוח QR</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>סים חדש ייעודי עדיף — לא לשבת על מספר קיים כי זה מנתק אותו</v>
       </c>
     </row>
     <row r="25">
@@ -1044,16 +1044,16 @@
         <v>7.5</v>
       </c>
       <c r="D25" t="str">
-        <v>התראות עיקבון לגבייה</v>
+        <v>שירות — FIXUS</v>
       </c>
       <c r="E25" t="str">
-        <v>בוצע</v>
+        <v>ממתין ללקוח</v>
       </c>
       <c r="F25" t="str">
-        <v>בכל פרויקט יש שדה "עיקבון (חודשים)" בכותרת. כשהפרויקט עובר ל"הושלם" — נוצרת משימה אוטומטית לרבקה עם תאריך יעד לפי תקופת העיקבון. גם 12 חודשים, גם 24 — הכל עובד.</v>
+        <v>בדקנו: ל-FIXUS יש API. הדומיין של ארגמן: arg-ac.fixus.co.il</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>יניר — להתקשר ל-FIXUS (052-8928581) ולבקש תיעוד API + מפתח גישה</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1070,19 +1070,19 @@
         <v>7.5</v>
       </c>
       <c r="D26" t="str">
-        <v>משימות קבועות בוואטסאפ</v>
+        <v>אקסלים של רבקה</v>
       </c>
       <c r="E26" t="str">
-        <v>טרם בוצע</v>
+        <v>ממתין ללקוח</v>
       </c>
       <c r="F26" t="str">
-        <v>משימות חוזרות חודשיות לאנשים ספציפיים.</v>
+        <v>לבנות ממשק במערכת במקום אקסלים.</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>רבקה — לשלוח את האקסלים</v>
       </c>
       <c r="H26" t="str">
-        <v>תלוי בחיבור וואטסאפ</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1093,27 +1093,79 @@
         <v>טליה</v>
       </c>
       <c r="C27" t="str">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="D27" t="str">
+        <v>בקשות תשלום ממותגות</v>
+      </c>
+      <c r="E27" t="str">
+        <v>לבדוק עם יניר</v>
+      </c>
+      <c r="F27" t="str">
+        <v>שליחת בקשת תשלום עם לוגו ללקוח. אולי לא רלוונטי כי יש מודול גבייה.</v>
+      </c>
+      <c r="G27" t="str">
+        <v>יניר — צריך את זה?</v>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C28" t="str">
+        <v>7.5</v>
+      </c>
+      <c r="D28" t="str">
+        <v>משימות קבועות בוואטסאפ</v>
+      </c>
+      <c r="E28" t="str">
+        <v>טרם בוצע</v>
+      </c>
+      <c r="F28" t="str">
+        <v>משימות חוזרות חודשיות לאנשים ספציפיים.</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v>תלוי בחיבור וואטסאפ (סעיף 23)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>טליה</v>
+      </c>
+      <c r="C29" t="str">
+        <v>8.5</v>
+      </c>
+      <c r="D29" t="str">
         <v>שינוי לוגיקת כתב כמויות</v>
       </c>
-      <c r="E27" t="str">
+      <c r="E29" t="str">
         <v>טרם בוצע</v>
       </c>
-      <c r="F27" t="str">
+      <c r="F29" t="str">
         <v>טבלה אחת (לא טאבים), כל החשבונות בעמודות. אושר ע"י טליה.</v>
       </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
-      <c r="H27" t="str">
-        <v/>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v>שינוי גדול — לתאם מתי</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>